<commit_message>
Sessão 17 (v2.9): Diagnóstico ML + Treinamento em Tempo Real
- Adicionadas 50 amostras metafóricas ao dataset (2050 total)
- Modelo retreinado: DDoS/Phishing agora classificados corretamente
- Endpoint SSE /train-stream no Flask com 8 passos em tempo real
- Proxy SSE /api/ml-train-stream no servidor Express
- Página AdminMLTraining.tsx com barra de progresso e métricas ao vivo
- Aviso de baixa confiança (< 40%) no IncidentDetail
- 41 novos testes S17 — total: 844 testes em 21 arquivos
</commit_message>
<xml_diff>
--- a/ml/incidentes_cybersecurity_2000.xlsx
+++ b/ml/incidentes_cybersecurity_2000.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="incidentes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2001"/>
+  <dimension ref="A1:C2051"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34433,6 +34433,856 @@
         </is>
       </c>
     </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>A Arte da Manipulação Psicológica</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr">
+        <is>
+          <t>técnicas de engenharia social para manipular psicologicamente usuários e obter credenciais de acesso através de mensagens falsas</t>
+        </is>
+      </c>
+      <c r="C2002" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
+          <t>O Pescador de Senhas</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr">
+        <is>
+          <t>ataque de phishing utilizando iscas digitais para capturar senhas e dados pessoais de usuários desatentos</t>
+        </is>
+      </c>
+      <c r="C2003" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>A Isca Digital</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>email fraudulento com link malicioso disfarçado de comunicação legítima para roubar credenciais de acesso</t>
+        </is>
+      </c>
+      <c r="C2004" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>O Espelho Enganoso</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>página falsa que imita site legítimo para capturar login e senha de usuários através de engenharia social</t>
+        </is>
+      </c>
+      <c r="C2005" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>Armadilha de Confiança</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>mensagem fraudulenta explorando confiança do usuário para obter dados sensíveis e credenciais bancárias</t>
+        </is>
+      </c>
+      <c r="C2006" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>O Lobo em Pele de Cordeiro</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>email malicioso disfarçado de comunicação oficial solicitando atualização de dados e senha de acesso</t>
+        </is>
+      </c>
+      <c r="C2007" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>A Teia da Ilusão</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>campanha de phishing com múltiplos vetores de engenharia social para capturar credenciais corporativas</t>
+        </is>
+      </c>
+      <c r="C2008" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>Engenharia do Engano</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>ataque sofisticado de engenharia social manipulando psicologicamente funcionários para revelar senhas e acessos</t>
+        </is>
+      </c>
+      <c r="C2009" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>O Truque do Mágico Digital</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>fraude por email com link de phishing redirecionando para página falsa que rouba dados de login</t>
+        </is>
+      </c>
+      <c r="C2010" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>Sedução Eletrônica</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>mensagem fraudulenta com apelo emocional para induzir usuário a clicar em link malicioso e fornecer senha</t>
+        </is>
+      </c>
+      <c r="C2011" t="inlineStr">
+        <is>
+          <t>phishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>O Estrangulamento da Disponibilidade</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>ataque que sobrecarrega servidores com volume massivo de requisições para tornar serviços indisponíveis para usuários legítimos</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>A Inundação Digital</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>ataque de negação de serviço distribuído inundando a rede com tráfego excessivo e tornando o servidor indisponível</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>O Colapso da Rede</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>sobrecarga intencional de requisições simultâneas causando colapso dos servidores e indisponibilidade do sistema</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>Tempestade de Pacotes</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>ataque ddos com tempestade de pacotes de rede sobrecarregando a infraestrutura e causando indisponibilidade</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>O Sufocamento do Servidor</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>ataque volumétrico que sufoca o servidor com tráfego anormal impedindo acesso de usuários legítimos ao serviço</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>Avalanche de Requisições</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>avalanche de requisições simultâneas de múltiplas origens sobrecarregando o servidor e causando negação de serviço</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>O Silenciamento dos Serviços</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>ataque distribuído de negação de serviço silenciando sistemas críticos através de sobrecarga de tráfego de rede</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>Paralisia da Infraestrutura</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>ataque ddos causando paralisia total da infraestrutura de rede com volume anormal de tráfego e requisições</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>O Bloqueio Total</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>bloqueio total de acesso ao servidor por sobrecarga intencional de requisições distribuídas de múltiplas origens</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>Saturação dos Recursos</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>saturação completa dos recursos do servidor por tráfego anormal causando indisponibilidade e negação de serviço</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr">
+        <is>
+          <t>ddos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>O Invasor Silencioso</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>malware instalado silenciosamente no sistema executando código malicioso em segundo plano sem conhecimento do usuário</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>A Sombra no Sistema</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>software malicioso operando como sombra no sistema coletando dados e executando ações não autorizadas</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>O Parasita Digital</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>malware parasita instalado automaticamente que consome recursos do sistema e exfiltra dados confidenciais</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>Código das Trevas</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>código malicioso executável instalado automaticamente comprometendo o sistema e permitindo acesso remoto não autorizado</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>O Vírus Fantasma</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>vírus furtivo detectado pelo antivírus operando em modo oculto e modificando arquivos do sistema operacional</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>A Praga Eletrônica</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>malware se espalhando pela rede corporativa infectando múltiplos dispositivos e comprometendo dados sensíveis</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>O Espião Interno</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>spyware instalado automaticamente monitorando atividades do usuário e enviando dados para servidor externo malicioso</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>Contaminação do Sistema</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>contaminação por malware detectada pelo antivírus com arquivo executável suspeito instalado automaticamente no sistema</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>O Sequestro Digital</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>ransomware criptografando arquivos do sistema e exigindo resgate para restaurar acesso aos dados corporativos</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>A Bomba Relógio no Código</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>malware com gatilho temporal instalado silenciosamente aguardando data específica para executar ação maliciosa</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr">
+        <is>
+          <t>malware</t>
+        </is>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>O Martelo nas Senhas</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>ataque de força bruta com tentativas repetidas e sistemáticas de autenticação para descobrir senha de acesso</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>A Persistência do Atacante</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>tentativas sequenciais persistentes de login detectadas indicando ataque de força bruta nas credenciais do sistema</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>Bombardeio de Credenciais</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>bombardeio de tentativas de autenticação com credenciais variadas caracterizando ataque de brute force no sistema</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>O Dicionário do Invasor</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>ataque de dicionário com lista de senhas comuns tentando autenticação repetida até encontrar credencial válida</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>Força Bruta nas Portas</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>tentativas sequenciais de autenticação detectadas em múltiplas portas caracterizando ataque de força bruta sistemático</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>A Teimosa Invasão</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>conta bloqueada por excesso de tentativas de login falhadas indicando ataque de força bruta persistente</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>Chuva de Tentativas</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>chuva de tentativas de autenticação falhadas detectadas no sistema indicando ataque de brute force automatizado</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>O Quebrador de Cofres</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>ataque sistemático tentando múltiplas combinações de senha para quebrar autenticação e acessar sistema protegido</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>Assalto às Credenciais</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>assalto sistemático às credenciais com tentativas sequenciais de autenticação detectadas no servidor de login</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>A Insistência Maliciosa</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>tentativas repetidas e insistentes de autenticação falhadas bloqueando conta por excesso de erros de senha</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>brute force</t>
+        </is>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>A Fuga de Segredos</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>vazamento de dados confidenciais detectado com informações sensíveis expostas em repositório público sem autorização</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>O Rio de Dados Perdidos</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>fluxo de dados confidenciais vazando para fora da organização com informações sensíveis expostas indevidamente</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>Segredos à Mostra</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>dados sensíveis encontrados em local público com informações confidenciais expostas sem controle de acesso adequado</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>A Brecha no Cofre</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>brecha de segurança permitindo acesso não autorizado a dados confidenciais com risco de vazamento de informações</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>O Vazamento Silencioso</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>exfiltração silenciosa de dados confidenciais detectada com informações sensíveis sendo enviadas para destino externo</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>Informações à Deriva</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>informações confidenciais à deriva na internet após vazamento de banco de dados acessado indevidamente</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>A Torneira Aberta</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>dados fluindo sem controle para fora da organização com arquivos internos compartilhados sem autorização adequada</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>O Espalhamento dos Dados</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>espalhamento não autorizado de dados confidenciais com informações sensíveis expostas em múltiplos locais públicos</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>Memória Exposta</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>dados sensíveis expostos em memória acessível publicamente com risco de vazamento de informações confidenciais</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>A Janela Aberta</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>janela de segurança aberta permitindo acesso não autorizado a dados confidenciais e vazamento de informações sensíveis</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>vazamento de dados</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>